<commit_message>
Add subscription plans and Stripe integration setup
</commit_message>
<xml_diff>
--- a/test_bank.xlsx
+++ b/test_bank.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,7 +417,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:D28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -436,264 +436,495 @@
           <t>description</t>
         </is>
       </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>type</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>45680</v>
+        <v>45681</v>
       </c>
       <c r="B2" t="n">
-        <v>2988.13</v>
+        <v>-2139.3</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Transaction 1</t>
+          <t>Consulting fee - Client XYZ</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>45679</v>
+        <v>45695</v>
       </c>
       <c r="B3" t="n">
-        <v>1808.85</v>
+        <v>1647.73</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Transaction 2</t>
+          <t>Salary payment</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>45679</v>
+        <v>45665</v>
       </c>
       <c r="B4" t="n">
-        <v>3296.42</v>
+        <v>-3373.84</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Transaction 3</t>
+          <t>Software license - Monthly</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>45679</v>
+        <v>45671</v>
       </c>
       <c r="B5" t="n">
-        <v>3420.76</v>
+        <v>-946.2</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Transaction 4</t>
+          <t>Office supplies - Stationery</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>45673</v>
+        <v>45677</v>
       </c>
       <c r="B6" t="n">
-        <v>359.82</v>
+        <v>-3759.97</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Transaction 5</t>
+          <t>Salary payment</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>45673</v>
+        <v>45662</v>
       </c>
       <c r="B7" t="n">
-        <v>3545.83</v>
+        <v>4100.74</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Transaction 6</t>
+          <t>Office supplies - Stationery</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>45671</v>
+        <v>45696</v>
       </c>
       <c r="B8" t="n">
-        <v>1877.64</v>
+        <v>3609</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Transaction 7</t>
+          <t>Travel reimbursement</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>45674</v>
+        <v>45691</v>
       </c>
       <c r="B9" t="n">
-        <v>1767.48</v>
+        <v>-1830.02</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Transaction 8</t>
+          <t>Dividend received</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>45687</v>
+        <v>45675</v>
       </c>
       <c r="B10" t="n">
-        <v>4306.98</v>
+        <v>-3603.1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Transaction 9</t>
+          <t>Interest earned</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
-        <v>45685</v>
+        <v>45694</v>
       </c>
       <c r="B11" t="n">
-        <v>2617.92</v>
+        <v>3734.43</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Transaction 10</t>
+          <t>Transfer to supplier - ABC Ltd</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="n">
-        <v>45672</v>
+        <v>45696</v>
       </c>
       <c r="B12" t="n">
-        <v>3659.02</v>
+        <v>1977.11</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Transaction 11</t>
+          <t>Consulting fee - Client XYZ</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="n">
-        <v>45666</v>
+        <v>45660</v>
       </c>
       <c r="B13" t="n">
-        <v>3584.72</v>
+        <v>1878.04</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Transaction 12</t>
+          <t>Client payment - Invoice #1234</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
-        <v>45684</v>
+        <v>45659</v>
       </c>
       <c r="B14" t="n">
-        <v>968.16</v>
+        <v>728</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Transaction 13</t>
+          <t>Rent payment - Office</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
-        <v>45666</v>
+        <v>45665</v>
       </c>
       <c r="B15" t="n">
-        <v>3631.12</v>
+        <v>3292.61</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Transaction 14</t>
+          <t>Interest earned</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
-        <v>45677</v>
+        <v>45662</v>
       </c>
       <c r="B16" t="n">
-        <v>3227.13</v>
+        <v>-2129.46</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Transaction 15</t>
+          <t>Software license - Monthly</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
-        <v>45686</v>
+        <v>45666</v>
       </c>
       <c r="B17" t="n">
-        <v>673.83</v>
+        <v>822.66</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Transaction 16</t>
+          <t>Salary payment</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
-        <v>45673</v>
+        <v>45668</v>
       </c>
       <c r="B18" t="n">
-        <v>640.15</v>
+        <v>3492.15</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Transaction 17</t>
+          <t>Travel reimbursement</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1" t="n">
-        <v>45661</v>
+        <v>45662</v>
       </c>
       <c r="B19" t="n">
-        <v>4229.85</v>
+        <v>856.92</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Transaction 18</t>
+          <t>Salary payment</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
-        <v>45668</v>
+        <v>45675</v>
       </c>
       <c r="B20" t="n">
-        <v>1840.75</v>
+        <v>-2595.21</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Transaction 19</t>
+          <t>Bank charges - Monthly fee</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>debit</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="1" t="n">
-        <v>45674</v>
+        <v>45694</v>
       </c>
       <c r="B21" t="n">
-        <v>2977.21</v>
+        <v>-4001.24</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Transaction 20</t>
+          <t>Rent payment - Office</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>debit</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="1" t="n">
+        <v>45686</v>
+      </c>
+      <c r="B22" t="n">
+        <v>-3182.58</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Insurance premium</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>debit</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="1" t="n">
+        <v>45668</v>
+      </c>
+      <c r="B23" t="n">
+        <v>2102.31</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Travel reimbursement</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="1" t="n">
+        <v>45665</v>
+      </c>
+      <c r="B24" t="n">
+        <v>2251.38</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Interest earned</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="1" t="n">
+        <v>45664</v>
+      </c>
+      <c r="B25" t="n">
+        <v>467.73</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>ATM withdrawal - Main branch</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>credit</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="1" t="n">
+        <v>45667</v>
+      </c>
+      <c r="B26" t="n">
+        <v>150.41</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Duplicate payment #3</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>debit</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="n">
+        <v>45662</v>
+      </c>
+      <c r="B27" t="n">
+        <v>-4494.61</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Software license - Monthly</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>debit</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="1" t="n">
+        <v>45694</v>
+      </c>
+      <c r="B28" t="n">
+        <v>3607.89</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Travel reimbursement</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>credit</t>
         </is>
       </c>
     </row>

</xml_diff>